<commit_message>
outputting hbars for country capacities
</commit_message>
<xml_diff>
--- a/reconcile/storage/output/capacities_plot.xlsx
+++ b/reconcile/storage/output/capacities_plot.xlsx
@@ -23389,7 +23389,7 @@
         <v>0.4</v>
       </c>
       <c r="M448" s="2" t="n">
-        <v>44287</v>
+        <v>45323</v>
       </c>
       <c r="N448" s="2" t="n">
         <v>44197</v>
@@ -23450,7 +23450,7 @@
         <v>0.4</v>
       </c>
       <c r="M449" s="2" t="n">
-        <v>44287</v>
+        <v>45323</v>
       </c>
       <c r="N449" s="2" t="n">
         <v>44197</v>
@@ -23928,9 +23928,7 @@
       <c r="L458" t="n">
         <v>0.4</v>
       </c>
-      <c r="M458" s="2" t="n">
-        <v>44287</v>
-      </c>
+      <c r="M458" t="inlineStr"/>
       <c r="N458" s="2" t="n">
         <v>44197</v>
       </c>
@@ -23985,9 +23983,7 @@
       <c r="L459" t="n">
         <v>0.4</v>
       </c>
-      <c r="M459" s="2" t="n">
-        <v>44287</v>
-      </c>
+      <c r="M459" t="inlineStr"/>
       <c r="N459" s="2" t="n">
         <v>44197</v>
       </c>

</xml_diff>